<commit_message>
chore: full backup fund tracking and earnings snapshot
</commit_message>
<xml_diff>
--- a/artifacts/fund_tracking/天弘全球新能源汽车QDII_LOF_164212_持仓跟踪.xlsx
+++ b/artifacts/fund_tracking/天弘全球新能源汽车QDII_LOF_164212_持仓跟踪.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="估算使用说明" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="说明" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="持仓明细" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="资产配置" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="地区行业" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="对比摘要" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="后续跟踪模板" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="重点观察标的" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="默认估算持仓" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="估算模型校验" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="估算使用说明" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="持仓明细" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="资产配置" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="地区行业" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="对比摘要" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="后续跟踪模板" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="重点观察标的" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="默认估算持仓" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="估算模型校验" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'说明'!$A$1:$B$10</definedName>
@@ -223,13 +223,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -253,7 +253,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -277,7 +277,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -305,8 +305,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -332,8 +332,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -359,7 +359,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>6</col>
@@ -374,9 +374,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 20:09:15</t>
+          <t>2026-06-28 20:15:12</t>
         </is>
       </c>
     </row>
@@ -1391,7 +1391,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11至2026-06-17：A份额累计+8.22%，C份额累计+8.22%；已追加日度拟合。</t>
+          <t>2026-06-18至2026-06-25：A份额累计+5.93%，C份额累计+5.92%；Q1可见持仓+CSOP估算约+2.05%，误差-3.87pct。</t>
         </is>
       </c>
     </row>
@@ -1403,7 +1403,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>截至本次运行，天天基金公告接口最新定期报告仍为2026年第1季度报告（2026-04-22，AN202604211821382912）；无新增季报/半年报/年报。</t>
+          <t>截至2026-06-28，天天基金/东方财富定期报告接口最新仍为天弘全球新能源汽车股票型证券投资基金(QDII-LOF)2026年第1季度报告（2026-04-22，AN202604211821382912）；未发现新的季报、半年报或年报。</t>
         </is>
       </c>
     </row>
@@ -1415,7 +1415,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>使用2026Q1前十大股票及CSOP 07709.HK、07747.HK可见权重，叠加Yahoo历史价格与USD/CNY、HKD/CNY；季度报告非全持仓披露。</t>
+          <t>使用2026Q1前十大股票及CSOP 07709.HK、07747.HK/09747.HK可见权重（合计约41.15%），叠加Yahoo历史价格与USD/CNY、HKD/CNY；季度报告非全量权益持仓披露。</t>
         </is>
       </c>
     </row>
@@ -8881,7 +8881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9215,6 +9215,266 @@
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>ttskill NAV + Yahoo chart + USD/CNY/HKD/CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>164212</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>2.5966</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>2.572</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>-2.22</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>KLAC/TSM/TER/7709.HK</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>LITE</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>可见Q1持仓方向与公布净值一致，但强度不足；缺口来自未披露持仓、调仓、杠杆或时点差异。</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>ttskill NAV + Yahoo chart + USD/CNY/HKD/CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>164212</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>2.6711</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>2.6457</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>2.87</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>-1.48</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>7709.HK/COHR/LITE/LRCX</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>AVGO/NVDA/7747.HK</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>可见Q1持仓方向与公布净值一致，但强度不足；缺口来自未披露持仓、调仓、杠杆或时点差异。</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>ttskill NAV + Yahoo chart + USD/CNY/HKD/CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>164212</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>2.4823</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>2.4587</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>-7.07</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>-3.41</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>3.66</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>无明显可见重仓正贡献</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>7709.HK/COHR/KLAC/7747.HK</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>可见AI链与两只CSOP 2x同步回撤；公布跌幅更深，提示未披露仓位或调仓放大下行。</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>ttskill NAV + Yahoo chart + USD/CNY/HKD/CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>164212</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>2.5392</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>2.5151</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>-1.63</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>7747.HK/7709.HK/COHR/LITE</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>KLAC/TSLA/NVDA</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>可见Q1持仓方向与公布净值一致，但强度不足；缺口来自未披露持仓、调仓、杠杆或时点差异。</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>ttskill NAV + Yahoo chart + USD/CNY/HKD/CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>164212</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>2.6419</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>2.6167</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>-2.44</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>7709.HK/TER/KLAC/LRCX</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>NVDA/TSM/AVGO/TSLA</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>可见Q1持仓方向与公布净值一致，但强度不足；缺口来自未披露持仓、调仓、杠杆或时点差异。</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>ttskill NAV + Yahoo chart + USD/CNY/HKD/CNY</t>
         </is>

</xml_diff>

<commit_message>
chore: full backup 2026-07-05 tracking updates
</commit_message>
<xml_diff>
--- a/artifacts/fund_tracking/天弘全球新能源汽车QDII_LOF_164212_持仓跟踪.xlsx
+++ b/artifacts/fund_tracking/天弘全球新能源汽车QDII_LOF_164212_持仓跟踪.xlsx
@@ -1283,7 +1283,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28 20:15:12</t>
+          <t>2026-07-05 20:10:38</t>
         </is>
       </c>
     </row>
@@ -1391,7 +1391,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18至2026-06-25：A份额累计+5.93%，C份额累计+5.92%；Q1可见持仓+CSOP估算约+2.05%，误差-3.87pct。</t>
+          <t>2026-06-26至2026-07-02：A份额累计-11.51%，C份额累计-11.51%；Q1前十大+CSOP可见仓位估算约-4.45%，误差+7.05pct（估算跌幅不足）。</t>
         </is>
       </c>
     </row>
@@ -1403,7 +1403,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>截至2026-06-28，天天基金/东方财富定期报告接口最新仍为天弘全球新能源汽车股票型证券投资基金(QDII-LOF)2026年第1季度报告（2026-04-22，AN202604211821382912）；未发现新的季报、半年报或年报。</t>
+          <t>截至2026-07-05，天天基金/东方财富定期报告接口最新仍为天弘全球新能源汽车股票型证券投资基金(QDII-LOF)2026年第1季度报告（2026-04-22，AN202604211821382912）；未发现新的季报、半年报或年报。</t>
         </is>
       </c>
     </row>
@@ -1415,7 +1415,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>使用2026Q1前十大股票及CSOP 07709.HK、07747.HK/09747.HK可见权重（合计约41.15%），叠加Yahoo历史价格与USD/CNY、HKD/CNY；季度报告非全量权益持仓披露。</t>
+          <t>使用2026Q1前十大股票及CSOP 07709.HK、07747.HK/09747.HK可见权重（合计约41.15%），叠加Yahoo历史价格与USD/CNY、HKD/CNY；港股休市日以前值填充；季度报告非全量权益持仓披露。</t>
         </is>
       </c>
     </row>
@@ -8881,7 +8881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9475,6 +9475,266 @@
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>ttskill NAV + Yahoo chart + USD/CNY/HKD/CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>164212</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>2.5284</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>2.5043</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>-4.3</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>-1.76</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>7709.HK/TER/COHR/LITE</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>可见AI硬件链与CSOP 2x同步回撤，但公布跌幅更深；缺口来自未披露持仓、调仓、估值或时点差异。</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>ttskill NAV + Yahoo chart + USD/CNY/HKD/CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>164212</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>2.5988</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>2.574</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>-1.06</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>KLAC/TSLA/LRCX/TER</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>7709.HK/7747.HK</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>美股AI硬件链反弹，CSOP 2x继续拖累；估算低于公布涨幅。</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>ttskill NAV + Yahoo chart + USD/CNY/HKD/CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>164212</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>2.6734</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>2.6478</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>2.87</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>-1.33</v>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>KLAC/AMD/TSM/LRCX</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>无明显可见重仓拖累</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Q1可见AI链普涨，方向与公布净值一致但强度不足。</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>ttskill NAV + Yahoo chart + USD/CNY/HKD/CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>164212</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>2.5612</v>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>2.5367</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>-4.2</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>-2.31</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>TER/KLAC/LRCX/TSM</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>港股7月1日休市，CSOP按前值处理；美股半导体设备和光通信回撤主导。</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>ttskill NAV + Yahoo chart + USD/CNY/HKD/CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>164212</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>2.3379</v>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>2.3155</v>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>-8.720000000000001</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>-3.61</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>5.11</v>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>无明显可见重仓正贡献</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>7709.HK/TER/KLAC/LITE</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>可见AI链与两只CSOP 2x大幅回撤，但公布跌幅明显更深；提示未披露仓位、调仓或估值时点差异显著。</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>ttskill NAV + Yahoo chart + USD/CNY/HKD/CNY</t>
         </is>

</xml_diff>